<commit_message>
Refresh site data assets
</commit_message>
<xml_diff>
--- a/data/FR.xlsx
+++ b/data/FR.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1561"/>
+  <dimension ref="A1:T1570"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63729,58 +63729,58 @@
         <v>1</v>
       </c>
       <c r="C1048" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D1048" t="n">
-        <v>-2.142857142857143</v>
+        <v>-2.285714285714286</v>
       </c>
       <c r="E1048" t="n">
-        <v>-1.866666666666667</v>
+        <v>-1.9</v>
       </c>
       <c r="F1048" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G1048" t="n">
         <v>0</v>
       </c>
       <c r="H1048" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I1048" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J1048" t="n">
         <v>0</v>
       </c>
       <c r="K1048" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L1048" t="n">
-        <v>-2</v>
+        <v>-2.333333333333333</v>
       </c>
       <c r="M1048" t="n">
         <v>-0.6666666666666666</v>
       </c>
       <c r="N1048" t="n">
-        <v>-0.3333333333333333</v>
+        <v>-0.6666666666666666</v>
       </c>
       <c r="O1048" t="n">
-        <v>-2.142857142857143</v>
+        <v>-2.285714285714286</v>
       </c>
       <c r="P1048" t="n">
         <v>-0.7142857142857143</v>
       </c>
       <c r="Q1048" t="n">
-        <v>-0.7142857142857143</v>
+        <v>-0.8571428571428571</v>
       </c>
       <c r="R1048" t="n">
-        <v>-1.866666666666667</v>
+        <v>-1.9</v>
       </c>
       <c r="S1048" t="n">
         <v>-0.2666666666666666</v>
       </c>
       <c r="T1048" t="n">
-        <v>-0.7333333333333333</v>
+        <v>-0.7666666666666667</v>
       </c>
     </row>
     <row r="1049">
@@ -63794,49 +63794,49 @@
       </c>
       <c r="C1049" t="inlineStr"/>
       <c r="D1049" t="n">
-        <v>-2.142857142857143</v>
+        <v>-2.428571428571428</v>
       </c>
       <c r="E1049" t="n">
-        <v>-1.8</v>
+        <v>-1.866666666666667</v>
       </c>
       <c r="F1049" t="inlineStr"/>
       <c r="G1049" t="inlineStr"/>
       <c r="H1049" t="inlineStr"/>
       <c r="I1049" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J1049" t="n">
         <v>0</v>
       </c>
       <c r="K1049" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L1049" t="n">
-        <v>-1</v>
+        <v>-1.666666666666667</v>
       </c>
       <c r="M1049" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="N1049" t="n">
-        <v>1.333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="O1049" t="n">
-        <v>-2.142857142857143</v>
+        <v>-2.428571428571428</v>
       </c>
       <c r="P1049" t="n">
         <v>-0.7142857142857143</v>
       </c>
       <c r="Q1049" t="n">
-        <v>-0.5714285714285714</v>
+        <v>-0.8571428571428571</v>
       </c>
       <c r="R1049" t="n">
-        <v>-1.8</v>
+        <v>-1.866666666666667</v>
       </c>
       <c r="S1049" t="n">
         <v>-0.2666666666666666</v>
       </c>
       <c r="T1049" t="n">
-        <v>-0.5666666666666667</v>
+        <v>-0.6333333333333333</v>
       </c>
     </row>
     <row r="1050">
@@ -63850,49 +63850,49 @@
       </c>
       <c r="C1050" t="inlineStr"/>
       <c r="D1050" t="n">
-        <v>-1.714285714285714</v>
+        <v>-2.142857142857143</v>
       </c>
       <c r="E1050" t="n">
-        <v>-1.733333333333333</v>
+        <v>-1.833333333333333</v>
       </c>
       <c r="F1050" t="inlineStr"/>
       <c r="G1050" t="inlineStr"/>
       <c r="H1050" t="inlineStr"/>
       <c r="I1050" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J1050" t="n">
         <v>0</v>
       </c>
       <c r="K1050" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L1050" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="M1050" t="n">
         <v>0</v>
       </c>
       <c r="N1050" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1050" t="n">
-        <v>-1.714285714285714</v>
+        <v>-2.142857142857143</v>
       </c>
       <c r="P1050" t="n">
         <v>-0.5714285714285714</v>
       </c>
       <c r="Q1050" t="n">
-        <v>0.1428571428571428</v>
+        <v>-0.2857142857142857</v>
       </c>
       <c r="R1050" t="n">
-        <v>-1.733333333333333</v>
+        <v>-1.833333333333333</v>
       </c>
       <c r="S1050" t="n">
         <v>-0.2666666666666666</v>
       </c>
       <c r="T1050" t="n">
-        <v>-0.4666666666666667</v>
+        <v>-0.5666666666666667</v>
       </c>
     </row>
     <row r="1051">
@@ -63908,10 +63908,10 @@
         <v>-2</v>
       </c>
       <c r="D1051" t="n">
-        <v>-1.571428571428571</v>
+        <v>-2</v>
       </c>
       <c r="E1051" t="n">
-        <v>-1.766666666666667</v>
+        <v>-1.866666666666667</v>
       </c>
       <c r="F1051" t="n">
         <v>-2</v>
@@ -63932,31 +63932,31 @@
         <v>-2</v>
       </c>
       <c r="L1051" t="n">
-        <v>-0.6666666666666666</v>
+        <v>-1.333333333333333</v>
       </c>
       <c r="M1051" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="N1051" t="n">
-        <v>1.333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="O1051" t="n">
-        <v>-1.571428571428571</v>
+        <v>-2</v>
       </c>
       <c r="P1051" t="n">
         <v>-0.5714285714285714</v>
       </c>
       <c r="Q1051" t="n">
-        <v>0.1428571428571428</v>
+        <v>-0.2857142857142857</v>
       </c>
       <c r="R1051" t="n">
-        <v>-1.766666666666667</v>
+        <v>-1.866666666666667</v>
       </c>
       <c r="S1051" t="n">
         <v>-0.3</v>
       </c>
       <c r="T1051" t="n">
-        <v>-0.5</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="1052">
@@ -63970,10 +63970,10 @@
       </c>
       <c r="C1052" t="inlineStr"/>
       <c r="D1052" t="n">
-        <v>-1.428571428571429</v>
+        <v>-1.857142857142857</v>
       </c>
       <c r="E1052" t="n">
-        <v>-1.766666666666667</v>
+        <v>-1.866666666666667</v>
       </c>
       <c r="F1052" t="inlineStr"/>
       <c r="G1052" t="inlineStr"/>
@@ -63988,31 +63988,31 @@
         <v>-2</v>
       </c>
       <c r="L1052" t="n">
-        <v>-1.333333333333333</v>
+        <v>-1.666666666666667</v>
       </c>
       <c r="M1052" t="n">
         <v>-0.6666666666666666</v>
       </c>
       <c r="N1052" t="n">
-        <v>-0.3333333333333333</v>
+        <v>-0.6666666666666666</v>
       </c>
       <c r="O1052" t="n">
-        <v>-1.428571428571429</v>
+        <v>-1.857142857142857</v>
       </c>
       <c r="P1052" t="n">
         <v>-0.5714285714285714</v>
       </c>
       <c r="Q1052" t="n">
-        <v>0.1428571428571428</v>
+        <v>-0.2857142857142857</v>
       </c>
       <c r="R1052" t="n">
-        <v>-1.766666666666667</v>
+        <v>-1.866666666666667</v>
       </c>
       <c r="S1052" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="T1052" t="n">
-        <v>-0.5333333333333333</v>
+        <v>-0.6333333333333333</v>
       </c>
     </row>
     <row r="1053">
@@ -64026,10 +64026,10 @@
       </c>
       <c r="C1053" t="inlineStr"/>
       <c r="D1053" t="n">
-        <v>-1.285714285714286</v>
+        <v>-1.714285714285714</v>
       </c>
       <c r="E1053" t="n">
-        <v>-1.766666666666667</v>
+        <v>-1.866666666666667</v>
       </c>
       <c r="F1053" t="inlineStr"/>
       <c r="G1053" t="inlineStr"/>
@@ -64053,22 +64053,22 @@
         <v>-2</v>
       </c>
       <c r="O1053" t="n">
-        <v>-1.285714285714286</v>
+        <v>-1.714285714285714</v>
       </c>
       <c r="P1053" t="n">
         <v>-0.5714285714285714</v>
       </c>
       <c r="Q1053" t="n">
-        <v>0.1428571428571428</v>
+        <v>-0.2857142857142857</v>
       </c>
       <c r="R1053" t="n">
-        <v>-1.766666666666667</v>
+        <v>-1.866666666666667</v>
       </c>
       <c r="S1053" t="n">
         <v>-0.3666666666666666</v>
       </c>
       <c r="T1053" t="n">
-        <v>-0.5333333333333333</v>
+        <v>-0.6333333333333333</v>
       </c>
     </row>
     <row r="1054">
@@ -64084,10 +64084,10 @@
         <v>-3</v>
       </c>
       <c r="D1054" t="n">
-        <v>-1.285714285714286</v>
+        <v>-1.714285714285714</v>
       </c>
       <c r="E1054" t="n">
-        <v>-1.8</v>
+        <v>-1.9</v>
       </c>
       <c r="F1054" t="n">
         <v>-3</v>
@@ -64117,22 +64117,22 @@
         <v>-1.333333333333333</v>
       </c>
       <c r="O1054" t="n">
-        <v>-1.285714285714286</v>
+        <v>-1.714285714285714</v>
       </c>
       <c r="P1054" t="n">
         <v>-0.4285714285714285</v>
       </c>
       <c r="Q1054" t="n">
-        <v>0.4285714285714285</v>
+        <v>0</v>
       </c>
       <c r="R1054" t="n">
-        <v>-1.8</v>
+        <v>-1.9</v>
       </c>
       <c r="S1054" t="n">
         <v>-0.3666666666666666</v>
       </c>
       <c r="T1054" t="n">
-        <v>-0.4666666666666667</v>
+        <v>-0.5666666666666667</v>
       </c>
     </row>
     <row r="1055">
@@ -64146,10 +64146,10 @@
       </c>
       <c r="C1055" t="inlineStr"/>
       <c r="D1055" t="n">
-        <v>-1.714285714285714</v>
+        <v>-2</v>
       </c>
       <c r="E1055" t="n">
-        <v>-1.833333333333333</v>
+        <v>-1.933333333333333</v>
       </c>
       <c r="F1055" t="inlineStr"/>
       <c r="G1055" t="inlineStr"/>
@@ -64173,22 +64173,22 @@
         <v>-0.6666666666666666</v>
       </c>
       <c r="O1055" t="n">
-        <v>-1.714285714285714</v>
+        <v>-2</v>
       </c>
       <c r="P1055" t="n">
         <v>-0.4285714285714285</v>
       </c>
       <c r="Q1055" t="n">
-        <v>0</v>
+        <v>-0.2857142857142857</v>
       </c>
       <c r="R1055" t="n">
-        <v>-1.833333333333333</v>
+        <v>-1.933333333333333</v>
       </c>
       <c r="S1055" t="n">
         <v>-0.3666666666666666</v>
       </c>
       <c r="T1055" t="n">
-        <v>-0.4</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="1056">
@@ -64204,10 +64204,10 @@
         <v>-2</v>
       </c>
       <c r="D1056" t="n">
-        <v>-2</v>
+        <v>-2.142857142857143</v>
       </c>
       <c r="E1056" t="n">
-        <v>-1.833333333333333</v>
+        <v>-1.933333333333333</v>
       </c>
       <c r="F1056" t="n">
         <v>-2</v>
@@ -64237,22 +64237,22 @@
         <v>-0.6666666666666666</v>
       </c>
       <c r="O1056" t="n">
-        <v>-2</v>
+        <v>-2.142857142857143</v>
       </c>
       <c r="P1056" t="n">
         <v>-0.4285714285714285</v>
       </c>
       <c r="Q1056" t="n">
-        <v>-0.7142857142857143</v>
+        <v>-0.8571428571428571</v>
       </c>
       <c r="R1056" t="n">
-        <v>-1.833333333333333</v>
+        <v>-1.933333333333333</v>
       </c>
       <c r="S1056" t="n">
         <v>-0.3666666666666666</v>
       </c>
       <c r="T1056" t="n">
-        <v>-0.4</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="1057">
@@ -64271,7 +64271,7 @@
         <v>-2.285714285714286</v>
       </c>
       <c r="E1057" t="n">
-        <v>-1.833333333333333</v>
+        <v>-1.933333333333333</v>
       </c>
       <c r="F1057" t="n">
         <v>-2</v>
@@ -64310,13 +64310,13 @@
         <v>-1.285714285714286</v>
       </c>
       <c r="R1057" t="n">
-        <v>-1.833333333333333</v>
+        <v>-1.933333333333333</v>
       </c>
       <c r="S1057" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="T1057" t="n">
-        <v>-0.3666666666666666</v>
+        <v>-0.4666666666666667</v>
       </c>
     </row>
     <row r="1058">
@@ -64335,7 +64335,7 @@
         <v>-2.428571428571428</v>
       </c>
       <c r="E1058" t="n">
-        <v>-1.866666666666667</v>
+        <v>-1.966666666666666</v>
       </c>
       <c r="F1058" t="n">
         <v>-3</v>
@@ -64374,13 +64374,13 @@
         <v>-1.285714285714286</v>
       </c>
       <c r="R1058" t="n">
-        <v>-1.866666666666667</v>
+        <v>-1.966666666666666</v>
       </c>
       <c r="S1058" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="T1058" t="n">
-        <v>-0.3666666666666666</v>
+        <v>-0.4666666666666667</v>
       </c>
     </row>
     <row r="1059">
@@ -64399,7 +64399,7 @@
         <v>-2.428571428571428</v>
       </c>
       <c r="E1059" t="n">
-        <v>-1.866666666666667</v>
+        <v>-1.966666666666666</v>
       </c>
       <c r="F1059" t="n">
         <v>-2</v>
@@ -64438,13 +64438,13 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="R1059" t="n">
-        <v>-1.866666666666667</v>
+        <v>-1.966666666666666</v>
       </c>
       <c r="S1059" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="T1059" t="n">
-        <v>-0.4666666666666667</v>
+        <v>-0.5666666666666667</v>
       </c>
     </row>
     <row r="1060">
@@ -64463,7 +64463,7 @@
         <v>-2.428571428571428</v>
       </c>
       <c r="E1060" t="n">
-        <v>-1.866666666666667</v>
+        <v>-1.966666666666666</v>
       </c>
       <c r="F1060" t="n">
         <v>-2</v>
@@ -64502,13 +64502,13 @@
         <v>-0.5714285714285714</v>
       </c>
       <c r="R1060" t="n">
-        <v>-1.866666666666667</v>
+        <v>-1.966666666666666</v>
       </c>
       <c r="S1060" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="T1060" t="n">
-        <v>-0.3666666666666666</v>
+        <v>-0.4666666666666667</v>
       </c>
     </row>
     <row r="1061">
@@ -64527,7 +64527,7 @@
         <v>-2</v>
       </c>
       <c r="E1061" t="n">
-        <v>-1.8</v>
+        <v>-1.9</v>
       </c>
       <c r="F1061" t="n">
         <v>0</v>
@@ -64566,13 +64566,13 @@
         <v>-0.4285714285714285</v>
       </c>
       <c r="R1061" t="n">
-        <v>-1.8</v>
+        <v>-1.9</v>
       </c>
       <c r="S1061" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="T1061" t="n">
-        <v>-0.3</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="1062">
@@ -64591,7 +64591,7 @@
         <v>-1.571428571428571</v>
       </c>
       <c r="E1062" t="n">
-        <v>-1.733333333333333</v>
+        <v>-1.833333333333333</v>
       </c>
       <c r="F1062" t="n">
         <v>0</v>
@@ -64630,13 +64630,13 @@
         <v>-0.4285714285714285</v>
       </c>
       <c r="R1062" t="n">
-        <v>-1.733333333333333</v>
+        <v>-1.833333333333333</v>
       </c>
       <c r="S1062" t="n">
         <v>-0.4</v>
       </c>
       <c r="T1062" t="n">
-        <v>-0.2666666666666666</v>
+        <v>-0.3666666666666666</v>
       </c>
     </row>
     <row r="1063">
@@ -64655,7 +64655,7 @@
         <v>-1.285714285714286</v>
       </c>
       <c r="E1063" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="F1063" t="n">
         <v>0</v>
@@ -64694,13 +64694,13 @@
         <v>0</v>
       </c>
       <c r="R1063" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="S1063" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="T1063" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="1064">
@@ -64719,7 +64719,7 @@
         <v>-1.285714285714286</v>
       </c>
       <c r="E1064" t="n">
-        <v>-1.633333333333333</v>
+        <v>-1.733333333333333</v>
       </c>
       <c r="F1064" t="n">
         <v>-2</v>
@@ -64758,13 +64758,13 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="R1064" t="n">
-        <v>-1.633333333333333</v>
+        <v>-1.733333333333333</v>
       </c>
       <c r="S1064" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="T1064" t="n">
-        <v>-0.1333333333333333</v>
+        <v>-0.2333333333333333</v>
       </c>
     </row>
     <row r="1065">
@@ -64781,7 +64781,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="E1065" t="n">
-        <v>-1.6</v>
+        <v>-1.7</v>
       </c>
       <c r="F1065" t="inlineStr"/>
       <c r="G1065" t="inlineStr"/>
@@ -64814,13 +64814,13 @@
         <v>0.4285714285714285</v>
       </c>
       <c r="R1065" t="n">
-        <v>-1.6</v>
+        <v>-1.7</v>
       </c>
       <c r="S1065" t="n">
         <v>-0.3333333333333333</v>
       </c>
       <c r="T1065" t="n">
-        <v>-0.0666666666666666</v>
+        <v>-0.1666666666666666</v>
       </c>
     </row>
     <row r="1066">
@@ -64837,7 +64837,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="E1066" t="n">
-        <v>-1.566666666666667</v>
+        <v>-1.666666666666667</v>
       </c>
       <c r="F1066" t="inlineStr"/>
       <c r="G1066" t="inlineStr"/>
@@ -64870,13 +64870,13 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="R1066" t="n">
-        <v>-1.566666666666667</v>
+        <v>-1.666666666666667</v>
       </c>
       <c r="S1066" t="n">
         <v>-0.4</v>
       </c>
       <c r="T1066" t="n">
-        <v>-0.0666666666666666</v>
+        <v>-0.1666666666666666</v>
       </c>
     </row>
     <row r="1067">
@@ -64895,7 +64895,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="E1067" t="n">
-        <v>-1.533333333333333</v>
+        <v>-1.633333333333333</v>
       </c>
       <c r="F1067" t="n">
         <v>-2</v>
@@ -64934,13 +64934,13 @@
         <v>0.4285714285714285</v>
       </c>
       <c r="R1067" t="n">
-        <v>-1.533333333333333</v>
+        <v>-1.633333333333333</v>
       </c>
       <c r="S1067" t="n">
         <v>-0.4</v>
       </c>
       <c r="T1067" t="n">
-        <v>-0.0333333333333333</v>
+        <v>-0.1333333333333333</v>
       </c>
     </row>
     <row r="1068">
@@ -64959,7 +64959,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="E1068" t="n">
-        <v>-1.6</v>
+        <v>-1.7</v>
       </c>
       <c r="F1068" t="n">
         <v>-2</v>
@@ -64998,13 +64998,13 @@
         <v>0.4285714285714285</v>
       </c>
       <c r="R1068" t="n">
-        <v>-1.6</v>
+        <v>-1.7</v>
       </c>
       <c r="S1068" t="n">
         <v>-0.4</v>
       </c>
       <c r="T1068" t="n">
-        <v>-0.0666666666666666</v>
+        <v>-0.1666666666666666</v>
       </c>
     </row>
     <row r="1069">
@@ -65023,7 +65023,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="E1069" t="n">
-        <v>-1.6</v>
+        <v>-1.7</v>
       </c>
       <c r="F1069" t="n">
         <v>0</v>
@@ -65062,13 +65062,13 @@
         <v>0.7142857142857143</v>
       </c>
       <c r="R1069" t="n">
-        <v>-1.6</v>
+        <v>-1.7</v>
       </c>
       <c r="S1069" t="n">
         <v>-0.4</v>
       </c>
       <c r="T1069" t="n">
-        <v>-0.0666666666666666</v>
+        <v>-0.1666666666666666</v>
       </c>
     </row>
     <row r="1070">
@@ -65087,7 +65087,7 @@
         <v>-1.571428571428571</v>
       </c>
       <c r="E1070" t="n">
-        <v>-1.633333333333333</v>
+        <v>-1.733333333333333</v>
       </c>
       <c r="F1070" t="n">
         <v>-1</v>
@@ -65126,13 +65126,13 @@
         <v>0.2857142857142857</v>
       </c>
       <c r="R1070" t="n">
-        <v>-1.633333333333333</v>
+        <v>-1.733333333333333</v>
       </c>
       <c r="S1070" t="n">
         <v>-0.4</v>
       </c>
       <c r="T1070" t="n">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="1071">
@@ -65151,7 +65151,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="E1071" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="F1071" t="n">
         <v>-1</v>
@@ -65190,13 +65190,13 @@
         <v>-0.1428571428571428</v>
       </c>
       <c r="R1071" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="S1071" t="n">
         <v>-0.4666666666666667</v>
       </c>
       <c r="T1071" t="n">
-        <v>-0.2666666666666666</v>
+        <v>-0.3666666666666666</v>
       </c>
     </row>
     <row r="1072">
@@ -65215,7 +65215,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="E1072" t="n">
-        <v>-1.733333333333333</v>
+        <v>-1.833333333333333</v>
       </c>
       <c r="F1072" t="n">
         <v>-2</v>
@@ -65254,13 +65254,13 @@
         <v>-0.5714285714285714</v>
       </c>
       <c r="R1072" t="n">
-        <v>-1.733333333333333</v>
+        <v>-1.833333333333333</v>
       </c>
       <c r="S1072" t="n">
         <v>-0.5333333333333333</v>
       </c>
       <c r="T1072" t="n">
-        <v>-0.4333333333333333</v>
+        <v>-0.5333333333333333</v>
       </c>
     </row>
     <row r="1073">
@@ -65277,7 +65277,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="E1073" t="n">
-        <v>-1.7</v>
+        <v>-1.8</v>
       </c>
       <c r="F1073" t="inlineStr"/>
       <c r="G1073" t="inlineStr"/>
@@ -65310,13 +65310,13 @@
         <v>-1</v>
       </c>
       <c r="R1073" t="n">
-        <v>-1.7</v>
+        <v>-1.8</v>
       </c>
       <c r="S1073" t="n">
         <v>-0.5666666666666667</v>
       </c>
       <c r="T1073" t="n">
-        <v>-0.4666666666666667</v>
+        <v>-0.5666666666666667</v>
       </c>
     </row>
     <row r="1074">
@@ -65333,7 +65333,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="E1074" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="F1074" t="inlineStr"/>
       <c r="G1074" t="inlineStr"/>
@@ -65366,13 +65366,13 @@
         <v>-1.571428571428571</v>
       </c>
       <c r="R1074" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="S1074" t="n">
         <v>-0.6</v>
       </c>
       <c r="T1074" t="n">
-        <v>-0.5</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="1075">
@@ -65391,7 +65391,7 @@
         <v>-1.571428571428571</v>
       </c>
       <c r="E1075" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="F1075" t="n">
         <v>-3</v>
@@ -65430,13 +65430,13 @@
         <v>-2</v>
       </c>
       <c r="R1075" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="S1075" t="n">
         <v>-0.5666666666666667</v>
       </c>
       <c r="T1075" t="n">
-        <v>-0.5</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="1076">
@@ -65455,7 +65455,7 @@
         <v>-2</v>
       </c>
       <c r="E1076" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="F1076" t="n">
         <v>-3</v>
@@ -65494,13 +65494,13 @@
         <v>-2.142857142857143</v>
       </c>
       <c r="R1076" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="S1076" t="n">
         <v>-0.6</v>
       </c>
       <c r="T1076" t="n">
-        <v>-0.4</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="1077">
@@ -65519,7 +65519,7 @@
         <v>-2.142857142857143</v>
       </c>
       <c r="E1077" t="n">
-        <v>-1.633333333333333</v>
+        <v>-1.733333333333333</v>
       </c>
       <c r="F1077" t="n">
         <v>-2</v>
@@ -65558,13 +65558,13 @@
         <v>-1.571428571428571</v>
       </c>
       <c r="R1077" t="n">
-        <v>-1.633333333333333</v>
+        <v>-1.733333333333333</v>
       </c>
       <c r="S1077" t="n">
         <v>-0.5666666666666667</v>
       </c>
       <c r="T1077" t="n">
-        <v>-0.2666666666666666</v>
+        <v>-0.3666666666666666</v>
       </c>
     </row>
     <row r="1078">
@@ -65583,7 +65583,7 @@
         <v>-2.142857142857143</v>
       </c>
       <c r="E1078" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.733333333333333</v>
       </c>
       <c r="F1078" t="n">
         <v>-1</v>
@@ -65622,13 +65622,13 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="R1078" t="n">
-        <v>-1.666666666666667</v>
+        <v>-1.733333333333333</v>
       </c>
       <c r="S1078" t="n">
         <v>-0.5666666666666667</v>
       </c>
       <c r="T1078" t="n">
-        <v>-0.3666666666666666</v>
+        <v>-0.4333333333333333</v>
       </c>
     </row>
     <row r="1079">
@@ -65647,7 +65647,7 @@
         <v>-2.142857142857143</v>
       </c>
       <c r="E1079" t="n">
-        <v>-1.733333333333333</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="F1079" t="n">
         <v>-2</v>
@@ -65686,13 +65686,13 @@
         <v>-0.4285714285714285</v>
       </c>
       <c r="R1079" t="n">
-        <v>-1.733333333333333</v>
+        <v>-1.766666666666667</v>
       </c>
       <c r="S1079" t="n">
         <v>-0.5333333333333333</v>
       </c>
       <c r="T1079" t="n">
-        <v>-0.4</v>
+        <v>-0.4333333333333333</v>
       </c>
     </row>
     <row r="1080">
@@ -77817,16 +77817,16 @@
         <v>1</v>
       </c>
       <c r="C1280" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="D1280" t="n">
-        <v>-1.285714285714286</v>
+        <v>-1.571428571428571</v>
       </c>
       <c r="E1280" t="n">
-        <v>-1.1</v>
+        <v>-1.166666666666667</v>
       </c>
       <c r="F1280" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G1280" t="n">
         <v>0</v>
@@ -77835,7 +77835,7 @@
         <v>-2</v>
       </c>
       <c r="I1280" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="J1280" t="n">
         <v>0</v>
@@ -77844,7 +77844,7 @@
         <v>-2</v>
       </c>
       <c r="L1280" t="n">
-        <v>-1.333333333333333</v>
+        <v>-2</v>
       </c>
       <c r="M1280" t="n">
         <v>0</v>
@@ -77853,7 +77853,7 @@
         <v>0</v>
       </c>
       <c r="O1280" t="n">
-        <v>-1.285714285714286</v>
+        <v>-1.571428571428571</v>
       </c>
       <c r="P1280" t="n">
         <v>0</v>
@@ -77862,7 +77862,7 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="R1280" t="n">
-        <v>-1.1</v>
+        <v>-1.166666666666667</v>
       </c>
       <c r="S1280" t="n">
         <v>0.2333333333333333</v>
@@ -77884,10 +77884,10 @@
         <v>-2</v>
       </c>
       <c r="D1281" t="n">
-        <v>-1.285714285714286</v>
+        <v>-1.571428571428571</v>
       </c>
       <c r="E1281" t="n">
-        <v>-1.1</v>
+        <v>-1.166666666666667</v>
       </c>
       <c r="F1281" t="n">
         <v>-2</v>
@@ -77908,7 +77908,7 @@
         <v>-1</v>
       </c>
       <c r="L1281" t="n">
-        <v>-1.333333333333333</v>
+        <v>-2</v>
       </c>
       <c r="M1281" t="n">
         <v>0</v>
@@ -77917,7 +77917,7 @@
         <v>-0.6666666666666666</v>
       </c>
       <c r="O1281" t="n">
-        <v>-1.285714285714286</v>
+        <v>-1.571428571428571</v>
       </c>
       <c r="P1281" t="n">
         <v>0</v>
@@ -77926,7 +77926,7 @@
         <v>0.2857142857142857</v>
       </c>
       <c r="R1281" t="n">
-        <v>-1.1</v>
+        <v>-1.166666666666667</v>
       </c>
       <c r="S1281" t="n">
         <v>0.2333333333333333</v>
@@ -77948,10 +77948,10 @@
         <v>0</v>
       </c>
       <c r="D1282" t="n">
-        <v>-1.142857142857143</v>
+        <v>-1.428571428571429</v>
       </c>
       <c r="E1282" t="n">
-        <v>-1.166666666666667</v>
+        <v>-1.233333333333333</v>
       </c>
       <c r="F1282" t="n">
         <v>0</v>
@@ -77972,7 +77972,7 @@
         <v>0</v>
       </c>
       <c r="L1282" t="n">
-        <v>-0.6666666666666666</v>
+        <v>-1.333333333333333</v>
       </c>
       <c r="M1282" t="n">
         <v>-0.3333333333333333</v>
@@ -77981,7 +77981,7 @@
         <v>-1</v>
       </c>
       <c r="O1282" t="n">
-        <v>-1.142857142857143</v>
+        <v>-1.428571428571429</v>
       </c>
       <c r="P1282" t="n">
         <v>-0.1428571428571428</v>
@@ -77990,7 +77990,7 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="R1282" t="n">
-        <v>-1.166666666666667</v>
+        <v>-1.233333333333333</v>
       </c>
       <c r="S1282" t="n">
         <v>0.1666666666666666</v>
@@ -78010,10 +78010,10 @@
       </c>
       <c r="C1283" t="inlineStr"/>
       <c r="D1283" t="n">
-        <v>-1</v>
+        <v>-1.285714285714286</v>
       </c>
       <c r="E1283" t="n">
-        <v>-1.166666666666667</v>
+        <v>-1.233333333333333</v>
       </c>
       <c r="F1283" t="inlineStr"/>
       <c r="G1283" t="inlineStr"/>
@@ -78037,7 +78037,7 @@
         <v>-0.3333333333333333</v>
       </c>
       <c r="O1283" t="n">
-        <v>-1</v>
+        <v>-1.285714285714286</v>
       </c>
       <c r="P1283" t="n">
         <v>-0.2857142857142857</v>
@@ -78046,7 +78046,7 @@
         <v>0</v>
       </c>
       <c r="R1283" t="n">
-        <v>-1.166666666666667</v>
+        <v>-1.233333333333333</v>
       </c>
       <c r="S1283" t="n">
         <v>0.1333333333333333</v>
@@ -78066,10 +78066,10 @@
       </c>
       <c r="C1284" t="inlineStr"/>
       <c r="D1284" t="n">
-        <v>-0.8571428571428571</v>
+        <v>-1.142857142857143</v>
       </c>
       <c r="E1284" t="n">
-        <v>-1.1</v>
+        <v>-1.166666666666667</v>
       </c>
       <c r="F1284" t="inlineStr"/>
       <c r="G1284" t="inlineStr"/>
@@ -78093,7 +78093,7 @@
         <v>0</v>
       </c>
       <c r="O1284" t="n">
-        <v>-0.8571428571428571</v>
+        <v>-1.142857142857143</v>
       </c>
       <c r="P1284" t="n">
         <v>-0.4285714285714285</v>
@@ -78102,7 +78102,7 @@
         <v>-0.1428571428571428</v>
       </c>
       <c r="R1284" t="n">
-        <v>-1.1</v>
+        <v>-1.166666666666667</v>
       </c>
       <c r="S1284" t="n">
         <v>0.1</v>
@@ -78124,10 +78124,10 @@
         <v>0</v>
       </c>
       <c r="D1285" t="n">
-        <v>-0.5714285714285714</v>
+        <v>-0.8571428571428571</v>
       </c>
       <c r="E1285" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="F1285" t="n">
         <v>0</v>
@@ -78157,7 +78157,7 @@
         <v>-0.3333333333333333</v>
       </c>
       <c r="O1285" t="n">
-        <v>-0.5714285714285714</v>
+        <v>-0.8571428571428571</v>
       </c>
       <c r="P1285" t="n">
         <v>-0.4285714285714285</v>
@@ -78166,7 +78166,7 @@
         <v>-0.4285714285714285</v>
       </c>
       <c r="R1285" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="S1285" t="n">
         <v>0.0666666666666666</v>
@@ -78188,10 +78188,10 @@
         <v>-2</v>
       </c>
       <c r="D1286" t="n">
-        <v>-0.5714285714285714</v>
+        <v>-0.8571428571428571</v>
       </c>
       <c r="E1286" t="n">
-        <v>-1.1</v>
+        <v>-1.166666666666667</v>
       </c>
       <c r="F1286" t="n">
         <v>-2</v>
@@ -78221,7 +78221,7 @@
         <v>-0.6666666666666666</v>
       </c>
       <c r="O1286" t="n">
-        <v>-0.5714285714285714</v>
+        <v>-0.8571428571428571</v>
       </c>
       <c r="P1286" t="n">
         <v>-0.4285714285714285</v>
@@ -78230,7 +78230,7 @@
         <v>-0.7142857142857143</v>
       </c>
       <c r="R1286" t="n">
-        <v>-1.1</v>
+        <v>-1.166666666666667</v>
       </c>
       <c r="S1286" t="n">
         <v>0.0333333333333333</v>
@@ -78255,7 +78255,7 @@
         <v>-0.2857142857142857</v>
       </c>
       <c r="E1287" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="F1287" t="n">
         <v>2</v>
@@ -78294,7 +78294,7 @@
         <v>0</v>
       </c>
       <c r="R1287" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="S1287" t="n">
         <v>0.0333333333333333</v>
@@ -78319,7 +78319,7 @@
         <v>0</v>
       </c>
       <c r="E1288" t="n">
-        <v>-0.9666666666666668</v>
+        <v>-1.033333333333333</v>
       </c>
       <c r="F1288" t="n">
         <v>0</v>
@@ -78358,7 +78358,7 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="R1288" t="n">
-        <v>-0.9666666666666668</v>
+        <v>-1.033333333333333</v>
       </c>
       <c r="S1288" t="n">
         <v>-0.0333333333333333</v>
@@ -78383,7 +78383,7 @@
         <v>-0.2857142857142857</v>
       </c>
       <c r="E1289" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="F1289" t="n">
         <v>-2</v>
@@ -78422,7 +78422,7 @@
         <v>-0.2857142857142857</v>
       </c>
       <c r="R1289" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="S1289" t="n">
         <v>-0.1</v>
@@ -78445,7 +78445,7 @@
         <v>-0.5714285714285714</v>
       </c>
       <c r="E1290" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="F1290" t="inlineStr"/>
       <c r="G1290" t="inlineStr"/>
@@ -78478,7 +78478,7 @@
         <v>-0.7142857142857143</v>
       </c>
       <c r="R1290" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="S1290" t="n">
         <v>-0.2</v>
@@ -78501,7 +78501,7 @@
         <v>-0.8571428571428571</v>
       </c>
       <c r="E1291" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="F1291" t="inlineStr"/>
       <c r="G1291" t="inlineStr"/>
@@ -78534,7 +78534,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="R1291" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="S1291" t="n">
         <v>-0.2333333333333333</v>
@@ -78557,7 +78557,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="E1292" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="F1292" t="inlineStr"/>
       <c r="G1292" t="inlineStr"/>
@@ -78590,7 +78590,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="R1292" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="S1292" t="n">
         <v>-0.2666666666666666</v>
@@ -78615,7 +78615,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="E1293" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="F1293" t="n">
         <v>-2</v>
@@ -78654,7 +78654,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="R1293" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="S1293" t="n">
         <v>-0.3</v>
@@ -78677,7 +78677,7 @@
         <v>-1.714285714285714</v>
       </c>
       <c r="E1294" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="F1294" t="inlineStr"/>
       <c r="G1294" t="inlineStr"/>
@@ -78710,7 +78710,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="R1294" t="n">
-        <v>-1.066666666666667</v>
+        <v>-1.133333333333333</v>
       </c>
       <c r="S1294" t="n">
         <v>-0.3333333333333333</v>
@@ -78735,7 +78735,7 @@
         <v>-1.714285714285714</v>
       </c>
       <c r="E1295" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="F1295" t="n">
         <v>0</v>
@@ -78774,7 +78774,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="R1295" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="S1295" t="n">
         <v>-0.3333333333333333</v>
@@ -78797,7 +78797,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="E1296" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="F1296" t="inlineStr"/>
       <c r="G1296" t="inlineStr"/>
@@ -78830,7 +78830,7 @@
         <v>-0.4285714285714285</v>
       </c>
       <c r="R1296" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="S1296" t="n">
         <v>-0.3</v>
@@ -78853,7 +78853,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="E1297" t="n">
-        <v>-0.9333333333333332</v>
+        <v>-1</v>
       </c>
       <c r="F1297" t="inlineStr"/>
       <c r="G1297" t="inlineStr"/>
@@ -78886,7 +78886,7 @@
         <v>0.2857142857142857</v>
       </c>
       <c r="R1297" t="n">
-        <v>-0.9333333333333332</v>
+        <v>-1</v>
       </c>
       <c r="S1297" t="n">
         <v>-0.3</v>
@@ -78909,7 +78909,7 @@
         <v>-0.8571428571428571</v>
       </c>
       <c r="E1298" t="n">
-        <v>-0.8666666666666667</v>
+        <v>-0.9333333333333332</v>
       </c>
       <c r="F1298" t="inlineStr"/>
       <c r="G1298" t="inlineStr"/>
@@ -78942,7 +78942,7 @@
         <v>1</v>
       </c>
       <c r="R1298" t="n">
-        <v>-0.8666666666666667</v>
+        <v>-0.9333333333333332</v>
       </c>
       <c r="S1298" t="n">
         <v>-0.3</v>
@@ -78967,7 +78967,7 @@
         <v>-1</v>
       </c>
       <c r="E1299" t="n">
-        <v>-0.9</v>
+        <v>-0.9666666666666668</v>
       </c>
       <c r="F1299" t="n">
         <v>-3</v>
@@ -79006,7 +79006,7 @@
         <v>1.142857142857143</v>
       </c>
       <c r="R1299" t="n">
-        <v>-0.9</v>
+        <v>-0.9666666666666668</v>
       </c>
       <c r="S1299" t="n">
         <v>-0.3</v>
@@ -79031,7 +79031,7 @@
         <v>-0.7142857142857143</v>
       </c>
       <c r="E1300" t="n">
-        <v>-0.9333333333333332</v>
+        <v>-1</v>
       </c>
       <c r="F1300" t="n">
         <v>0</v>
@@ -79070,7 +79070,7 @@
         <v>1.142857142857143</v>
       </c>
       <c r="R1300" t="n">
-        <v>-0.9333333333333332</v>
+        <v>-1</v>
       </c>
       <c r="S1300" t="n">
         <v>-0.3666666666666666</v>
@@ -79095,7 +79095,7 @@
         <v>-0.1428571428571428</v>
       </c>
       <c r="E1301" t="n">
-        <v>-0.9</v>
+        <v>-0.9666666666666668</v>
       </c>
       <c r="F1301" t="n">
         <v>2</v>
@@ -79134,7 +79134,7 @@
         <v>1.285714285714286</v>
       </c>
       <c r="R1301" t="n">
-        <v>-0.9</v>
+        <v>-0.9666666666666668</v>
       </c>
       <c r="S1301" t="n">
         <v>-0.3333333333333333</v>
@@ -79159,7 +79159,7 @@
         <v>-0.4285714285714285</v>
       </c>
       <c r="E1302" t="n">
-        <v>-0.9</v>
+        <v>-0.9666666666666668</v>
       </c>
       <c r="F1302" t="n">
         <v>-2</v>
@@ -79198,7 +79198,7 @@
         <v>1.142857142857143</v>
       </c>
       <c r="R1302" t="n">
-        <v>-0.9</v>
+        <v>-0.9666666666666668</v>
       </c>
       <c r="S1302" t="n">
         <v>-0.3333333333333333</v>
@@ -79221,7 +79221,7 @@
         <v>-0.7142857142857143</v>
       </c>
       <c r="E1303" t="n">
-        <v>-0.9333333333333332</v>
+        <v>-1</v>
       </c>
       <c r="F1303" t="inlineStr"/>
       <c r="G1303" t="inlineStr"/>
@@ -79254,7 +79254,7 @@
         <v>1</v>
       </c>
       <c r="R1303" t="n">
-        <v>-0.9333333333333332</v>
+        <v>-1</v>
       </c>
       <c r="S1303" t="n">
         <v>-0.3333333333333333</v>
@@ -79277,7 +79277,7 @@
         <v>-1</v>
       </c>
       <c r="E1304" t="n">
-        <v>-0.9333333333333332</v>
+        <v>-1</v>
       </c>
       <c r="F1304" t="inlineStr"/>
       <c r="G1304" t="inlineStr"/>
@@ -79310,7 +79310,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="R1304" t="n">
-        <v>-0.9333333333333332</v>
+        <v>-1</v>
       </c>
       <c r="S1304" t="n">
         <v>-0.3333333333333333</v>
@@ -79333,7 +79333,7 @@
         <v>-1.285714285714286</v>
       </c>
       <c r="E1305" t="n">
-        <v>-0.9666666666666668</v>
+        <v>-1.033333333333333</v>
       </c>
       <c r="F1305" t="inlineStr"/>
       <c r="G1305" t="inlineStr"/>
@@ -79366,7 +79366,7 @@
         <v>0.7142857142857143</v>
       </c>
       <c r="R1305" t="n">
-        <v>-0.9666666666666668</v>
+        <v>-1.033333333333333</v>
       </c>
       <c r="S1305" t="n">
         <v>-0.3333333333333333</v>
@@ -79391,7 +79391,7 @@
         <v>-1.142857142857143</v>
       </c>
       <c r="E1306" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="F1306" t="n">
         <v>-2</v>
@@ -79430,7 +79430,7 @@
         <v>1.285714285714286</v>
       </c>
       <c r="R1306" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="S1306" t="n">
         <v>-0.3333333333333333</v>
@@ -79455,7 +79455,7 @@
         <v>-1.428571428571429</v>
       </c>
       <c r="E1307" t="n">
-        <v>-1.033333333333333</v>
+        <v>-1.1</v>
       </c>
       <c r="F1307" t="n">
         <v>-2</v>
@@ -79494,7 +79494,7 @@
         <v>1.285714285714286</v>
       </c>
       <c r="R1307" t="n">
-        <v>-1.033333333333333</v>
+        <v>-1.1</v>
       </c>
       <c r="S1307" t="n">
         <v>-0.3333333333333333</v>
@@ -79519,7 +79519,7 @@
         <v>-1.714285714285714</v>
       </c>
       <c r="E1308" t="n">
-        <v>-0.9666666666666668</v>
+        <v>-1.033333333333333</v>
       </c>
       <c r="F1308" t="n">
         <v>0</v>
@@ -79558,7 +79558,7 @@
         <v>1.142857142857143</v>
       </c>
       <c r="R1308" t="n">
-        <v>-0.9666666666666668</v>
+        <v>-1.033333333333333</v>
       </c>
       <c r="S1308" t="n">
         <v>-0.3333333333333333</v>
@@ -79583,7 +79583,7 @@
         <v>-1.857142857142857</v>
       </c>
       <c r="E1309" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="F1309" t="n">
         <v>-3</v>
@@ -79622,7 +79622,7 @@
         <v>0.7142857142857143</v>
       </c>
       <c r="R1309" t="n">
-        <v>-1</v>
+        <v>-1.066666666666667</v>
       </c>
       <c r="S1309" t="n">
         <v>-0.3333333333333333</v>
@@ -95173,6 +95173,558 @@
       </c>
       <c r="T1561" t="n">
         <v>-0.2333333333333333</v>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1562" t="b">
+        <v>1</v>
+      </c>
+      <c r="C1562" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D1562" t="n">
+        <v>-0.1428571428571428</v>
+      </c>
+      <c r="E1562" t="n">
+        <v>-0.9333333333333332</v>
+      </c>
+      <c r="F1562" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G1562" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1562" t="n">
+        <v>1</v>
+      </c>
+      <c r="I1562" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J1562" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1562" t="n">
+        <v>1</v>
+      </c>
+      <c r="L1562" t="n">
+        <v>-0.3333333333333333</v>
+      </c>
+      <c r="M1562" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1562" t="n">
+        <v>1.666666666666667</v>
+      </c>
+      <c r="O1562" t="n">
+        <v>-0.1428571428571428</v>
+      </c>
+      <c r="P1562" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="Q1562" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="R1562" t="n">
+        <v>-0.9333333333333332</v>
+      </c>
+      <c r="S1562" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+      <c r="T1562" t="n">
+        <v>-0.1333333333333333</v>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1563" t="b">
+        <v>0</v>
+      </c>
+      <c r="C1563" t="inlineStr"/>
+      <c r="D1563" t="n">
+        <v>-0.4285714285714285</v>
+      </c>
+      <c r="E1563" t="n">
+        <v>-0.9666666666666668</v>
+      </c>
+      <c r="F1563" t="inlineStr"/>
+      <c r="G1563" t="inlineStr"/>
+      <c r="H1563" t="inlineStr"/>
+      <c r="I1563" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J1563" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1563" t="n">
+        <v>1</v>
+      </c>
+      <c r="L1563" t="n">
+        <v>-1</v>
+      </c>
+      <c r="M1563" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1563" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="O1563" t="n">
+        <v>-0.4285714285714285</v>
+      </c>
+      <c r="P1563" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="Q1563" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="R1563" t="n">
+        <v>-0.9666666666666668</v>
+      </c>
+      <c r="S1563" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+      <c r="T1563" t="n">
+        <v>-0.1666666666666666</v>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1564" t="b">
+        <v>0</v>
+      </c>
+      <c r="C1564" t="inlineStr"/>
+      <c r="D1564" t="n">
+        <v>-0.7142857142857143</v>
+      </c>
+      <c r="E1564" t="n">
+        <v>-0.9333333333333332</v>
+      </c>
+      <c r="F1564" t="inlineStr"/>
+      <c r="G1564" t="inlineStr"/>
+      <c r="H1564" t="inlineStr"/>
+      <c r="I1564" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J1564" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1564" t="n">
+        <v>1</v>
+      </c>
+      <c r="L1564" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M1564" t="n">
+        <v>0</v>
+      </c>
+      <c r="N1564" t="n">
+        <v>1</v>
+      </c>
+      <c r="O1564" t="n">
+        <v>-0.7142857142857143</v>
+      </c>
+      <c r="P1564" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="Q1564" t="n">
+        <v>1</v>
+      </c>
+      <c r="R1564" t="n">
+        <v>-0.9333333333333332</v>
+      </c>
+      <c r="S1564" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+      <c r="T1564" t="n">
+        <v>-0.0666666666666666</v>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1565" t="b">
+        <v>1</v>
+      </c>
+      <c r="C1565" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D1565" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E1565" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="F1565" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G1565" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1565" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1565" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J1565" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1565" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1565" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M1565" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N1565" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="O1565" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P1565" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="Q1565" t="n">
+        <v>1.285714285714286</v>
+      </c>
+      <c r="R1565" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="S1565" t="n">
+        <v>0.5666666666666667</v>
+      </c>
+      <c r="T1565" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1566">
+      <c r="A1566" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1566" t="b">
+        <v>1</v>
+      </c>
+      <c r="C1566" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D1566" t="n">
+        <v>-1.285714285714286</v>
+      </c>
+      <c r="E1566" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F1566" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G1566" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H1566" t="n">
+        <v>1</v>
+      </c>
+      <c r="I1566" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J1566" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K1566" t="n">
+        <v>1</v>
+      </c>
+      <c r="L1566" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M1566" t="n">
+        <v>0</v>
+      </c>
+      <c r="N1566" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="O1566" t="n">
+        <v>-1.285714285714286</v>
+      </c>
+      <c r="P1566" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="Q1566" t="n">
+        <v>1.142857142857143</v>
+      </c>
+      <c r="R1566" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S1566" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+      <c r="T1566" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1567" t="b">
+        <v>0</v>
+      </c>
+      <c r="C1567" t="inlineStr"/>
+      <c r="D1567" t="n">
+        <v>-1.571428571428571</v>
+      </c>
+      <c r="E1567" t="n">
+        <v>-1.166666666666667</v>
+      </c>
+      <c r="F1567" t="inlineStr"/>
+      <c r="G1567" t="inlineStr"/>
+      <c r="H1567" t="inlineStr"/>
+      <c r="I1567" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J1567" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K1567" t="n">
+        <v>1</v>
+      </c>
+      <c r="L1567" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M1567" t="n">
+        <v>-0.3333333333333333</v>
+      </c>
+      <c r="N1567" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="O1567" t="n">
+        <v>-1.571428571428571</v>
+      </c>
+      <c r="P1567" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="Q1567" t="n">
+        <v>1</v>
+      </c>
+      <c r="R1567" t="n">
+        <v>-1.166666666666667</v>
+      </c>
+      <c r="S1567" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="T1567" t="n">
+        <v>0.0333333333333333</v>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1568" t="b">
+        <v>1</v>
+      </c>
+      <c r="C1568" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D1568" t="n">
+        <v>-2.142857142857143</v>
+      </c>
+      <c r="E1568" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="F1568" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G1568" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H1568" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I1568" t="n">
+        <v>-3</v>
+      </c>
+      <c r="J1568" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K1568" t="n">
+        <v>-2</v>
+      </c>
+      <c r="L1568" t="n">
+        <v>-2.333333333333333</v>
+      </c>
+      <c r="M1568" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N1568" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1568" t="n">
+        <v>-2.142857142857143</v>
+      </c>
+      <c r="P1568" t="n">
+        <v>-0.2857142857142857</v>
+      </c>
+      <c r="Q1568" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="R1568" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="S1568" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="T1568" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B1569" t="b">
+        <v>1</v>
+      </c>
+      <c r="C1569" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1569" t="n">
+        <v>-1.857142857142857</v>
+      </c>
+      <c r="E1569" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="F1569" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1569" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1569" t="n">
+        <v>1</v>
+      </c>
+      <c r="I1569" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1569" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1569" t="n">
+        <v>1</v>
+      </c>
+      <c r="L1569" t="n">
+        <v>-1.666666666666667</v>
+      </c>
+      <c r="M1569" t="n">
+        <v>-0.6666666666666666</v>
+      </c>
+      <c r="N1569" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1569" t="n">
+        <v>-1.857142857142857</v>
+      </c>
+      <c r="P1569" t="n">
+        <v>-0.2857142857142857</v>
+      </c>
+      <c r="Q1569" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="R1569" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="S1569" t="n">
+        <v>0.3666666666666666</v>
+      </c>
+      <c r="T1569" t="n">
+        <v>-0.0333333333333333</v>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B1570" t="b">
+        <v>1</v>
+      </c>
+      <c r="C1570" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D1570" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E1570" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="F1570" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G1570" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1570" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1570" t="n">
+        <v>-3</v>
+      </c>
+      <c r="J1570" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1570" t="n">
+        <v>2</v>
+      </c>
+      <c r="L1570" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M1570" t="n">
+        <v>-0.3333333333333333</v>
+      </c>
+      <c r="N1570" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="O1570" t="n">
+        <v>-2</v>
+      </c>
+      <c r="P1570" t="n">
+        <v>-0.2857142857142857</v>
+      </c>
+      <c r="Q1570" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="R1570" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="S1570" t="n">
+        <v>0.3666666666666666</v>
+      </c>
+      <c r="T1570" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -95233,7 +95785,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Backward-compatible alias for c1_raw, the WDSI publication-day raw score.</t>
+          <t>Backward-compatible alias for c1_raw, the c1 publication-day raw score (war-related DSI / WDSI).</t>
         </is>
       </c>
     </row>
@@ -95245,7 +95797,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Backward-compatible alias for c1_7, the 7-day smoothed WDSI.</t>
+          <t>Backward-compatible alias for c1_7, the 7-day smoothed c1 series (war-related DSI / WDSI).</t>
         </is>
       </c>
     </row>
@@ -95257,7 +95809,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Backward-compatible alias for c1_30, the 30-day smoothed WDSI.</t>
+          <t>Backward-compatible alias for c1_30, the 30-day smoothed c1 series (war-related DSI / WDSI).</t>
         </is>
       </c>
     </row>

</xml_diff>